<commit_message>
finished EDA on the data, atleast for closure times
</commit_message>
<xml_diff>
--- a/facebook/data/manual_closure_or_reopening_times_finished.xlsx
+++ b/facebook/data/manual_closure_or_reopening_times_finished.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/hudson/Desktop/road_project/facebook/data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6B9EB497-272B-344C-8369-14513F08544C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DBB53E6E-3EF5-7042-A3E1-46605B6A94B0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="740" windowWidth="29400" windowHeight="16960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4964" uniqueCount="2865">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4966" uniqueCount="2867">
   <si>
     <t>Unnamed: 0</t>
   </si>
@@ -11441,7 +11441,13 @@
     <t>6/25/20 22:31 PM</t>
   </si>
   <si>
-    <t>03/16/19/4:53 PM</t>
+    <t>03/16/18/4:53 PM</t>
+  </si>
+  <si>
+    <t>w</t>
+  </si>
+  <si>
+    <t>5/5/2024  5:15AM</t>
   </si>
 </sst>
 </file>
@@ -11449,7 +11455,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd\ hh:mm:ss"/>
   </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
@@ -11491,7 +11497,7 @@
   </cellStyleXfs>
   <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -11804,6 +11810,7 @@
   <dimension ref="A1:V618"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
+    <col min="3" max="3" width="11.83203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="17.6640625" bestFit="1" customWidth="1"/>
     <col min="13" max="13" width="8.83203125" customWidth="1"/>
     <col min="14" max="14" width="50.83203125" style="3" customWidth="1"/>
@@ -13462,7 +13469,7 @@
         <v>132</v>
       </c>
       <c r="V25" s="4">
-        <v>45971.380555555559</v>
+        <v>45981.380555555559</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="192" x14ac:dyDescent="0.2">
@@ -16037,8 +16044,8 @@
       <c r="U65" t="s">
         <v>322</v>
       </c>
-      <c r="V65" s="4">
-        <v>46146.9375</v>
+      <c r="V65" s="4" t="s">
+        <v>2866</v>
       </c>
     </row>
     <row r="66" spans="1:22" ht="128" x14ac:dyDescent="0.2">
@@ -16171,7 +16178,7 @@
         <v>331</v>
       </c>
       <c r="V67" s="4">
-        <v>46146.791666666664</v>
+        <v>45416.791666666664</v>
       </c>
     </row>
     <row r="68" spans="1:22" ht="112" x14ac:dyDescent="0.2">
@@ -16369,7 +16376,7 @@
         <v>345</v>
       </c>
       <c r="V70" s="4">
-        <v>46104.315972222219</v>
+        <v>45374.315972222219</v>
       </c>
     </row>
     <row r="71" spans="1:22" ht="272" x14ac:dyDescent="0.2">
@@ -21468,7 +21475,7 @@
         <v>708</v>
       </c>
       <c r="V149" s="4">
-        <v>44940.104166666664</v>
+        <v>44941.104166666664</v>
       </c>
     </row>
     <row r="150" spans="1:22" ht="272" x14ac:dyDescent="0.2">
@@ -22948,7 +22955,7 @@
         <v>811</v>
       </c>
       <c r="V172" s="4">
-        <v>45261.491666666669</v>
+        <v>44896.491666666669</v>
       </c>
     </row>
     <row r="173" spans="1:22" ht="224" x14ac:dyDescent="0.2">
@@ -23264,7 +23271,7 @@
         <v>834</v>
       </c>
       <c r="V177" s="4">
-        <v>45604.801388888889</v>
+        <v>44873.915277777778</v>
       </c>
     </row>
     <row r="178" spans="1:22" ht="144" x14ac:dyDescent="0.2">
@@ -23332,7 +23339,7 @@
         <v>839</v>
       </c>
       <c r="V178" s="4">
-        <v>45604.801388888889</v>
+        <v>44873.801388888889</v>
       </c>
     </row>
     <row r="179" spans="1:22" ht="208" x14ac:dyDescent="0.2">
@@ -23831,7 +23838,7 @@
         <v>878</v>
       </c>
       <c r="V186" s="4">
-        <v>44823.802083333336</v>
+        <v>44823.885416666664</v>
       </c>
     </row>
     <row r="187" spans="1:22" ht="80" x14ac:dyDescent="0.2">
@@ -23958,7 +23965,7 @@
         <v>887</v>
       </c>
       <c r="V188" s="4">
-        <v>44823.25</v>
+        <v>44823.3125</v>
       </c>
     </row>
     <row r="189" spans="1:22" ht="192" x14ac:dyDescent="0.2">
@@ -24149,8 +24156,8 @@
       <c r="U191" t="s">
         <v>901</v>
       </c>
-      <c r="V191" s="4">
-        <v>44817.746527777781</v>
+      <c r="V191" s="4" t="s">
+        <v>2865</v>
       </c>
     </row>
     <row r="192" spans="1:22" ht="176" x14ac:dyDescent="0.2">
@@ -28828,9 +28835,7 @@
       <c r="U265" t="s">
         <v>1244</v>
       </c>
-      <c r="V265" s="4">
-        <v>44376.724999999999</v>
-      </c>
+      <c r="V265" s="4"/>
     </row>
     <row r="266" spans="1:22" ht="64" x14ac:dyDescent="0.2">
       <c r="A266">
@@ -34458,7 +34463,7 @@
         <v>1653</v>
       </c>
       <c r="V355" s="4">
-        <v>43796.325694444444</v>
+        <v>43796.375</v>
       </c>
     </row>
     <row r="356" spans="1:22" ht="380" x14ac:dyDescent="0.2">
@@ -34906,9 +34911,7 @@
       <c r="U362" t="s">
         <v>1685</v>
       </c>
-      <c r="V362" s="4">
-        <v>43736.75</v>
-      </c>
+      <c r="V362" s="4"/>
     </row>
     <row r="363" spans="1:22" ht="240" x14ac:dyDescent="0.2">
       <c r="A363">
@@ -37423,7 +37426,7 @@
         <v>1870</v>
       </c>
       <c r="V402" s="4">
-        <v>43517.352777777778</v>
+        <v>43517.365972222222</v>
       </c>
     </row>
     <row r="403" spans="1:22" ht="409.6" x14ac:dyDescent="0.2">
@@ -37932,7 +37935,7 @@
         <v>1906</v>
       </c>
       <c r="V410" s="4">
-        <v>43520.645833333336</v>
+        <v>43512.645833333336</v>
       </c>
     </row>
     <row r="411" spans="1:22" ht="380" x14ac:dyDescent="0.2">
@@ -39001,7 +39004,7 @@
         <v>1982</v>
       </c>
       <c r="V427" s="4">
-        <v>43501.260416666664</v>
+        <v>43501.411111111112</v>
       </c>
     </row>
     <row r="428" spans="1:22" ht="380" x14ac:dyDescent="0.2">
@@ -39066,7 +39069,7 @@
         <v>1986</v>
       </c>
       <c r="V428" s="4">
-        <v>43501.260416666664</v>
+        <v>43501.411111111112</v>
       </c>
     </row>
     <row r="429" spans="1:22" ht="48" x14ac:dyDescent="0.2">
@@ -39134,7 +39137,7 @@
         <v>1990</v>
       </c>
       <c r="V429" s="4">
-        <v>43501.260416666664</v>
+        <v>43501.411111111112</v>
       </c>
     </row>
     <row r="430" spans="1:22" ht="176" x14ac:dyDescent="0.2">
@@ -39199,7 +39202,7 @@
         <v>1995</v>
       </c>
       <c r="V430" s="4">
-        <v>43501.260416666664</v>
+        <v>43501.411111111112</v>
       </c>
     </row>
     <row r="431" spans="1:22" ht="320" x14ac:dyDescent="0.2">
@@ -39263,6 +39266,9 @@
       <c r="U431" t="s">
         <v>1999</v>
       </c>
+      <c r="V431" s="4">
+        <v>43501.411111111112</v>
+      </c>
     </row>
     <row r="432" spans="1:22" ht="64" x14ac:dyDescent="0.2">
       <c r="A432">
@@ -44966,7 +44972,7 @@
         <v>2415</v>
       </c>
       <c r="V522" s="4">
-        <v>43173.450694444444</v>
+        <v>43173.531944444447</v>
       </c>
     </row>
     <row r="523" spans="1:22" ht="192" x14ac:dyDescent="0.2">

</xml_diff>